<commit_message>
1016158: Modified template file
</commit_message>
<xml_diff>
--- a/Offer-Letter-Automation/Offer-Letter-Automation/wwwroot/Data/Data.xlsx
+++ b/Offer-Letter-Automation/Offer-Letter-Automation/wwwroot/Data/Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Blog\Offer-Letter\Offer-Letter-Automation\Offer-Letter-Automation\wwwroot\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Blog\OfferLetter-Usecase\Offer-Letter-Automation\Offer-Letter-Automation\wwwroot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73DE5E7-A6DC-4671-BFD6-58A3ECF145CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB1DE51-7F0E-46D0-9701-F2CC87F0CBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="136">
   <si>
     <t>OfferCode</t>
   </si>
@@ -98,9 +98,6 @@
     <t>RetirementPlan</t>
   </si>
   <si>
-    <t>TrainingBudget</t>
-  </si>
-  <si>
     <t>WorkArrangement</t>
   </si>
   <si>
@@ -110,9 +107,6 @@
     <t>NoticeRequired</t>
   </si>
   <si>
-    <t>NonCompetePeriod</t>
-  </si>
-  <si>
     <t>HREmail</t>
   </si>
   <si>
@@ -173,9 +167,6 @@
     <t>2 Months</t>
   </si>
   <si>
-    <t>12 Months</t>
-  </si>
-  <si>
     <t>hr@globaltech.co.uk</t>
   </si>
   <si>
@@ -225,9 +216,6 @@
   </si>
   <si>
     <t>1 Month</t>
-  </si>
-  <si>
-    <t>6 Months</t>
   </si>
   <si>
     <t>hr@technova.in</t>
@@ -818,7 +806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" customWidth="1"/>
@@ -842,16 +830,14 @@
     <col min="19" max="19" width="15.5546875" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="18.77734375" customWidth="1"/>
-    <col min="22" max="22" width="17.21875" customWidth="1"/>
-    <col min="23" max="23" width="16.6640625" customWidth="1"/>
-    <col min="24" max="24" width="16.33203125" customWidth="1"/>
-    <col min="25" max="25" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" customWidth="1"/>
+    <col min="23" max="23" width="16.33203125" customWidth="1"/>
+    <col min="24" max="24" width="16.6640625" customWidth="1"/>
+    <col min="25" max="25" width="18.33203125" customWidth="1"/>
     <col min="26" max="26" width="19.21875" customWidth="1"/>
-    <col min="27" max="27" width="18.33203125" customWidth="1"/>
-    <col min="28" max="28" width="19.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -877,7 +863,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -930,67 +916,61 @@
       <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="B2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>28</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>30</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>31</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>32</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" t="s">
         <v>33</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>34</v>
       </c>
-      <c r="I2" t="s">
-        <v>134</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>35</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" t="s">
         <v>36</v>
       </c>
-      <c r="L2" t="s">
+      <c r="O2" t="s">
         <v>37</v>
-      </c>
-      <c r="M2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" t="s">
-        <v>38</v>
-      </c>
-      <c r="O2" t="s">
-        <v>39</v>
       </c>
       <c r="P2">
         <v>75000</v>
       </c>
       <c r="Q2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="S2">
         <v>25</v>
@@ -999,84 +979,78 @@
         <v>10</v>
       </c>
       <c r="U2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V2" t="s">
+        <v>41</v>
+      </c>
+      <c r="W2">
+        <v>6</v>
+      </c>
+      <c r="X2" t="s">
         <v>42</v>
       </c>
-      <c r="V2">
-        <v>2000</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="Y2" t="s">
         <v>43</v>
       </c>
-      <c r="X2">
-        <v>6</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>44</v>
       </c>
-      <c r="Z2" t="s">
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>45</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="C3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
         <v>48</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" t="s">
         <v>49</v>
       </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>50</v>
       </c>
-      <c r="D3" t="s">
+      <c r="H3" t="s">
         <v>51</v>
       </c>
-      <c r="E3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
+        <v>133</v>
+      </c>
+      <c r="J3" t="s">
         <v>52</v>
       </c>
-      <c r="G3" t="s">
+      <c r="K3" t="s">
         <v>53</v>
       </c>
-      <c r="H3" t="s">
+      <c r="L3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" t="s">
+        <v>84</v>
+      </c>
+      <c r="N3" t="s">
+        <v>90</v>
+      </c>
+      <c r="O3" t="s">
         <v>54</v>
-      </c>
-      <c r="I3" t="s">
-        <v>137</v>
-      </c>
-      <c r="J3" t="s">
-        <v>55</v>
-      </c>
-      <c r="K3" t="s">
-        <v>56</v>
-      </c>
-      <c r="L3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s">
-        <v>88</v>
-      </c>
-      <c r="N3" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" t="s">
-        <v>57</v>
       </c>
       <c r="P3">
         <v>1200000</v>
       </c>
       <c r="Q3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="R3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="S3">
         <v>20</v>
@@ -1085,84 +1059,78 @@
         <v>12</v>
       </c>
       <c r="U3" t="s">
+        <v>57</v>
+      </c>
+      <c r="V3" t="s">
+        <v>58</v>
+      </c>
+      <c r="W3">
+        <v>3</v>
+      </c>
+      <c r="X3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y3" t="s">
         <v>60</v>
       </c>
-      <c r="V3">
-        <v>150000</v>
-      </c>
-      <c r="W3" t="s">
+      <c r="Z3" t="s">
         <v>61</v>
       </c>
-      <c r="X3">
-        <v>3</v>
-      </c>
-      <c r="Y3" t="s">
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>62</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="B4" t="s">
         <v>63</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="C4" t="s">
         <v>64</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="D4" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="E4" t="s">
         <v>66</v>
       </c>
-      <c r="B4" t="s">
+      <c r="F4" t="s">
         <v>67</v>
       </c>
-      <c r="C4" t="s">
+      <c r="G4" t="s">
         <v>68</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H4" t="s">
         <v>69</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
+        <v>134</v>
+      </c>
+      <c r="J4" t="s">
         <v>70</v>
       </c>
-      <c r="F4" t="s">
+      <c r="K4" t="s">
         <v>71</v>
       </c>
-      <c r="G4" t="s">
+      <c r="L4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" t="s">
+      <c r="M4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N4" t="s">
+        <v>66</v>
+      </c>
+      <c r="O4" t="s">
         <v>73</v>
-      </c>
-      <c r="I4" t="s">
-        <v>138</v>
-      </c>
-      <c r="J4" t="s">
-        <v>74</v>
-      </c>
-      <c r="K4" t="s">
-        <v>75</v>
-      </c>
-      <c r="L4" t="s">
-        <v>76</v>
-      </c>
-      <c r="M4" t="s">
-        <v>70</v>
-      </c>
-      <c r="N4" t="s">
-        <v>70</v>
-      </c>
-      <c r="O4" t="s">
-        <v>77</v>
       </c>
       <c r="P4">
         <v>42000</v>
       </c>
       <c r="Q4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="R4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="S4">
         <v>22</v>
@@ -1171,84 +1139,78 @@
         <v>8</v>
       </c>
       <c r="U4" t="s">
+        <v>76</v>
+      </c>
+      <c r="V4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W4">
+        <v>4</v>
+      </c>
+      <c r="X4" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>78</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>80</v>
       </c>
-      <c r="V4">
-        <v>1800</v>
-      </c>
-      <c r="W4" t="s">
+      <c r="B5" t="s">
         <v>81</v>
       </c>
-      <c r="X4">
-        <v>4</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA4" t="s">
+      <c r="C5" t="s">
         <v>82</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="D5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="E5" t="s">
         <v>84</v>
       </c>
-      <c r="B5" t="s">
+      <c r="F5" t="s">
         <v>85</v>
       </c>
-      <c r="C5" t="s">
+      <c r="G5" t="s">
         <v>86</v>
       </c>
-      <c r="D5" t="s">
+      <c r="H5" t="s">
         <v>87</v>
       </c>
-      <c r="E5" t="s">
+      <c r="I5" t="s">
+        <v>132</v>
+      </c>
+      <c r="J5" t="s">
         <v>88</v>
       </c>
-      <c r="F5" t="s">
+      <c r="K5" t="s">
         <v>89</v>
       </c>
-      <c r="G5" t="s">
+      <c r="L5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" t="s">
+        <v>84</v>
+      </c>
+      <c r="N5" t="s">
         <v>90</v>
       </c>
-      <c r="H5" t="s">
+      <c r="O5" t="s">
         <v>91</v>
-      </c>
-      <c r="I5" t="s">
-        <v>136</v>
-      </c>
-      <c r="J5" t="s">
-        <v>92</v>
-      </c>
-      <c r="K5" t="s">
-        <v>93</v>
-      </c>
-      <c r="L5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" t="s">
-        <v>88</v>
-      </c>
-      <c r="N5" t="s">
-        <v>94</v>
-      </c>
-      <c r="O5" t="s">
-        <v>95</v>
       </c>
       <c r="P5">
         <v>95000</v>
       </c>
       <c r="Q5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="R5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="S5">
         <v>18</v>
@@ -1257,84 +1219,78 @@
         <v>10</v>
       </c>
       <c r="U5" t="s">
+        <v>94</v>
+      </c>
+      <c r="V5" t="s">
+        <v>41</v>
+      </c>
+      <c r="W5">
+        <v>6</v>
+      </c>
+      <c r="X5" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>98</v>
       </c>
-      <c r="V5">
-        <v>2500</v>
-      </c>
-      <c r="W5" t="s">
-        <v>43</v>
-      </c>
-      <c r="X5">
-        <v>6</v>
-      </c>
-      <c r="Y5" t="s">
+      <c r="B6" t="s">
         <v>99</v>
       </c>
-      <c r="Z5" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA5" t="s">
+      <c r="C6" t="s">
         <v>100</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="D6" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="E6" t="s">
         <v>102</v>
       </c>
-      <c r="B6" t="s">
+      <c r="F6" t="s">
         <v>103</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
         <v>104</v>
       </c>
-      <c r="D6" t="s">
+      <c r="H6" t="s">
         <v>105</v>
       </c>
-      <c r="E6" t="s">
+      <c r="I6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J6" t="s">
         <v>106</v>
       </c>
-      <c r="F6" t="s">
+      <c r="K6" t="s">
         <v>107</v>
       </c>
-      <c r="G6" t="s">
+      <c r="L6" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" t="s">
+        <v>102</v>
+      </c>
+      <c r="N6" t="s">
+        <v>102</v>
+      </c>
+      <c r="O6" t="s">
         <v>108</v>
-      </c>
-      <c r="H6" t="s">
-        <v>109</v>
-      </c>
-      <c r="I6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J6" t="s">
-        <v>110</v>
-      </c>
-      <c r="K6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L6" t="s">
-        <v>37</v>
-      </c>
-      <c r="M6" t="s">
-        <v>106</v>
-      </c>
-      <c r="N6" t="s">
-        <v>106</v>
-      </c>
-      <c r="O6" t="s">
-        <v>112</v>
       </c>
       <c r="P6">
         <v>200000</v>
       </c>
       <c r="Q6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="S6">
         <v>15</v>
@@ -1343,84 +1299,78 @@
         <v>7</v>
       </c>
       <c r="U6" t="s">
+        <v>110</v>
+      </c>
+      <c r="V6" t="s">
+        <v>58</v>
+      </c>
+      <c r="W6">
+        <v>3</v>
+      </c>
+      <c r="X6" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" t="s">
         <v>114</v>
       </c>
-      <c r="V6">
-        <v>1200</v>
-      </c>
-      <c r="W6" t="s">
-        <v>61</v>
-      </c>
-      <c r="X6">
-        <v>3</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA6" t="s">
+      <c r="C7" t="s">
         <v>115</v>
       </c>
-      <c r="AB6" t="s">
+      <c r="D7" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="E7" t="s">
         <v>117</v>
       </c>
-      <c r="B7" t="s">
+      <c r="F7" t="s">
         <v>118</v>
       </c>
-      <c r="C7" t="s">
+      <c r="G7" t="s">
         <v>119</v>
       </c>
-      <c r="D7" t="s">
+      <c r="H7" t="s">
         <v>120</v>
       </c>
-      <c r="E7" t="s">
+      <c r="I7" t="s">
+        <v>135</v>
+      </c>
+      <c r="J7" t="s">
         <v>121</v>
       </c>
-      <c r="F7" t="s">
+      <c r="K7" t="s">
         <v>122</v>
       </c>
-      <c r="G7" t="s">
+      <c r="L7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" t="s">
+        <v>117</v>
+      </c>
+      <c r="N7" t="s">
         <v>123</v>
       </c>
-      <c r="H7" t="s">
+      <c r="O7" t="s">
         <v>124</v>
-      </c>
-      <c r="I7" t="s">
-        <v>139</v>
-      </c>
-      <c r="J7" t="s">
-        <v>125</v>
-      </c>
-      <c r="K7" t="s">
-        <v>126</v>
-      </c>
-      <c r="L7" t="s">
-        <v>37</v>
-      </c>
-      <c r="M7" t="s">
-        <v>121</v>
-      </c>
-      <c r="N7" t="s">
-        <v>127</v>
-      </c>
-      <c r="O7" t="s">
-        <v>128</v>
       </c>
       <c r="P7">
         <v>140000</v>
       </c>
       <c r="Q7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R7" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="S7">
         <v>30</v>
@@ -1429,28 +1379,22 @@
         <v>12</v>
       </c>
       <c r="U7" t="s">
-        <v>130</v>
-      </c>
-      <c r="V7">
-        <v>3000</v>
-      </c>
-      <c r="W7" t="s">
-        <v>43</v>
-      </c>
-      <c r="X7">
+        <v>126</v>
+      </c>
+      <c r="V7" t="s">
+        <v>41</v>
+      </c>
+      <c r="W7">
         <v>6</v>
       </c>
+      <c r="X7" t="s">
+        <v>59</v>
+      </c>
       <c r="Y7" t="s">
-        <v>62</v>
+        <v>127</v>
       </c>
       <c r="Z7" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>131</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>